<commit_message>
improve unit tests for show_intro and create_player
</commit_message>
<xml_diff>
--- a/docs/logbooks/riciano.xlsx
+++ b/docs/logbooks/riciano.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hrnl-my.sharepoint.com/personal/1101779_hr_nl/Documents/BaseCamp/Dossier Basecamp/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hrnl-my.sharepoint.com/personal/1101779_hr_nl/Documents/BaseCamp/DND_GAME/py-dnd-game/docs/logbooks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="58" documentId="8_{FD960573-718E-426B-9907-4B5AB4FC59EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A3346511-A492-49A3-8351-5A4D6A5ED29C}"/>
+  <xr:revisionPtr revIDLastSave="64" documentId="8_{FD960573-718E-426B-9907-4B5AB4FC59EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73ABAB82-DC07-48C6-87FF-0176589E4E8E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="37">
   <si>
     <t>🤔 Why keep a logbook?</t>
   </si>
@@ -217,6 +217,18 @@
   </si>
   <si>
     <t>Bezig met Level 2 van het verhaal en extra enemies toe te voegen en de story uit te breiden</t>
+  </si>
+  <si>
+    <t>Donderdag 14 Mei</t>
+  </si>
+  <si>
+    <t>Bezig met kijken hoe ik een Unittest moet gaan maken</t>
+  </si>
+  <si>
+    <t>Vrijdag 15 Mei</t>
+  </si>
+  <si>
+    <t>Unittest voor Show_intro() gemaakt en voor Create_Player()</t>
   </si>
 </sst>
 </file>
@@ -1753,7 +1765,7 @@
       </c>
       <c r="G4" s="12">
         <f>SUM(E4:E93)</f>
-        <v>0.62847222222222232</v>
+        <v>0.75347222222222232</v>
       </c>
     </row>
     <row r="5" spans="2:7" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.2">
@@ -1858,24 +1870,30 @@
       <c r="F10" s="17"/>
     </row>
     <row r="11" spans="2:7" s="13" customFormat="1" ht="15" x14ac:dyDescent="0.2">
-      <c r="B11" s="16"/>
+      <c r="B11" s="16" t="s">
+        <v>33</v>
+      </c>
       <c r="C11" s="17"/>
       <c r="D11" s="17"/>
       <c r="E11" s="22">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F11" s="17"/>
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="F11" s="17" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="12" spans="2:7" s="13" customFormat="1" ht="15" x14ac:dyDescent="0.2">
-      <c r="B12" s="16"/>
+      <c r="B12" s="16" t="s">
+        <v>35</v>
+      </c>
       <c r="C12" s="17"/>
       <c r="D12" s="17"/>
       <c r="E12" s="22">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F12" s="17"/>
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="F12" s="17" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="13" spans="2:7" s="13" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="B13" s="16"/>
@@ -5102,6 +5120,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ECB8076E25ECA940B4BF35F49653BD2F" ma:contentTypeVersion="3" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="9a8b4120c1d72a2dd47811016382667a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e8e5384f-6535-4009-8006-72859d350593" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="94add03b24b2efb618cd98e25f673028" ns2:_="">
     <xsd:import namespace="e8e5384f-6535-4009-8006-72859d350593"/>
@@ -5239,12 +5263,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{78E03D4F-D06B-40C1-A53D-F1DEB199C8A7}">
   <ds:schemaRefs>
@@ -5254,6 +5272,15 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14BB4D6E-C856-4503-A5F5-487F247D347A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7296CE53-CBBF-4225-9F98-E0028F76F8E2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5269,13 +5296,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14BB4D6E-C856-4503-A5F5-487F247D347A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>